<commit_message>
Rewrite all 248 scaffolds as genuine cloze statements with first-letter hints
Scaffolds now follow the pattern from the user's example:
- Definitions reversed: give the description, blank the term with first letter hint
  e.g. "A group of tissues working together is called an o_____."
- Short answers: statement context + first letter(s) of answer
  e.g. "The role of xylem tissue is to t_____ w_____ up through the plant."
- Lists: each item given first letter hint
  e.g. "The three blood vessel types are a_____, v_____ and c_____."

https://claude.ai/code/session_01GvPecmorJnDGHmg8pyuTjf
</commit_message>
<xml_diff>
--- a/data/questions-template.xlsx
+++ b/data/questions-template.xlsx
@@ -456,7 +456,7 @@
         <v>An organisms ability to get rid of waste</v>
       </c>
       <c r="I2" t="str">
-        <v>The 'E' in MRS GREN means _____.</v>
+        <v>The 'E' in MRS GREN stands for e_____: an organism's ability to get rid of waste.</v>
       </c>
     </row>
     <row r="3">
@@ -485,7 +485,7 @@
         <v>An organisms ability to grow in mass and height</v>
       </c>
       <c r="I3" t="str">
-        <v>The 'G' in MRS GREN means _____.</v>
+        <v>The 'G' in MRS GREN stands for g_____: an organism's ability to grow in mass and height.</v>
       </c>
     </row>
     <row r="4">
@@ -514,7 +514,7 @@
         <v>An organisms ability to move</v>
       </c>
       <c r="I4" t="str">
-        <v>The 'M' in MRS GREN means _____.</v>
+        <v>The 'M' in MRS GREN stands for m_____: an organism's ability to move.</v>
       </c>
     </row>
     <row r="5">
@@ -543,7 +543,7 @@
         <v>An organisms ability to get nutrients from food</v>
       </c>
       <c r="I5" t="str">
-        <v>The 'N' in MRS GREN means _____.</v>
+        <v>The 'N' in MRS GREN stands for n_____: an organism's ability to get nutrients from food.</v>
       </c>
     </row>
     <row r="6">
@@ -572,7 +572,7 @@
         <v>A group of tissues working together for specific functions</v>
       </c>
       <c r="I6" t="str">
-        <v>An organ is _____.</v>
+        <v>A group of tissues working together for a specific function is called an o_____.</v>
       </c>
     </row>
     <row r="7">
@@ -601,7 +601,7 @@
         <v>Absorb water and minerals from the soil</v>
       </c>
       <c r="I7" t="str">
-        <v>As well as anchoring the plant, roots also _____.</v>
+        <v>As well as holding the plant in place, roots also a_____ w_____ and m_____ from the soil.</v>
       </c>
     </row>
     <row r="8">
@@ -630,7 +630,7 @@
         <v>The leaf</v>
       </c>
       <c r="I8" t="str">
-        <v>The main organ of nutrition in a plant is _____.</v>
+        <v>The main organ of nutrition in a plant is the l_____.</v>
       </c>
     </row>
     <row r="9">
@@ -659,7 +659,7 @@
         <v>A group of cells with similar structure working together for a specific function</v>
       </c>
       <c r="I9" t="str">
-        <v>A tissue is _____.</v>
+        <v>A group of similar cells working together for a specific function is called a t_____.</v>
       </c>
     </row>
     <row r="10">
@@ -688,7 +688,7 @@
         <v>Muscle and fat (accept nerve as well)</v>
       </c>
       <c r="I10" t="str">
-        <v>Two tissues found in the heart are _____.</v>
+        <v>Two tissues found in the heart are m_____ and f_____.</v>
       </c>
     </row>
     <row r="11">
@@ -717,7 +717,7 @@
         <v>To transport water</v>
       </c>
       <c r="I11" t="str">
-        <v>The role of xylem tissue is _____.</v>
+        <v>The role of xylem tissue is to t_____ w_____ up through the plant.</v>
       </c>
     </row>
     <row r="12">
@@ -746,7 +746,7 @@
         <v>DNA contained in a nucleus</v>
       </c>
       <c r="I12" t="str">
-        <v>A eukaryotic cell is one where _____.</v>
+        <v>A cell that has its DNA contained within a nucleus is called a e_____ c_____.</v>
       </c>
     </row>
     <row r="13">
@@ -775,7 +775,7 @@
         <v>Lots of chloroplasts</v>
       </c>
       <c r="I13" t="str">
-        <v>An adaptation of a palisade cell is _____.</v>
+        <v>An adaptation of a palisade cell is having lots of c_____ to absorb light.</v>
       </c>
     </row>
     <row r="14">
@@ -804,7 +804,7 @@
         <v>Nucleus, cell membrane, ribosomes, cytoplasm, mitochondria</v>
       </c>
       <c r="I14" t="str">
-        <v>The 5 sub-cellular organelles in an animal cell are _____.</v>
+        <v>The 5 sub-cellular organelles in an animal cell: n_____, c_____ m_____, r_____, c_____ and m_____.</v>
       </c>
     </row>
     <row r="15">
@@ -833,7 +833,7 @@
         <v>Nucleus, cell membrane, ribosomes, cytoplasm, mitochondria, cell wall, chloroplast and vacuole</v>
       </c>
       <c r="I15" t="str">
-        <v>The 8 sub-cellular organelles in a plant cell are _____.</v>
+        <v>The 8 sub-cellular organelles in a plant cell: n_____, c_____ m_____, r_____, c_____, m_____, c_____ w_____, c_____ and v_____.</v>
       </c>
     </row>
     <row r="16">
@@ -862,7 +862,7 @@
         <v>Circulatory, nervous, muscular, respiratory, digestive, skeletal</v>
       </c>
       <c r="I16" t="str">
-        <v>Six organ systems found in the human body include _____.</v>
+        <v>The six organ systems in the body: c_____, n_____, m_____, r_____, d_____ and s_____.</v>
       </c>
     </row>
     <row r="17">
@@ -891,7 +891,7 @@
         <v>Cell &lt; Tissue &lt; Organ &lt; Organ system &lt; Organism</v>
       </c>
       <c r="I17" t="str">
-        <v>In order from smallest to largest: cell, tissue, organ, organ system, _____ is the largest.</v>
+        <v>From smallest to largest: cell &lt; t_____ &lt; o_____ &lt; o_____ s_____ &lt; organism.</v>
       </c>
     </row>
     <row r="18">
@@ -920,7 +920,7 @@
         <v>To transport substances around our body</v>
       </c>
       <c r="I18" t="str">
-        <v>The role of the circulatory system is _____.</v>
+        <v>The role of the circulatory system is to t_____ substances around the body.</v>
       </c>
     </row>
     <row r="19">
@@ -949,7 +949,7 @@
         <v>Nucleus of male and female sex cell joining</v>
       </c>
       <c r="I19" t="str">
-        <v>Fertilisation is _____.</v>
+        <v>The joining of the nuclei of a male and female sex cell is called f_____.</v>
       </c>
     </row>
     <row r="20">
@@ -978,7 +978,7 @@
         <v>Sex cells</v>
       </c>
       <c r="I20" t="str">
-        <v>A gamete is _____.</v>
+        <v>Sex cells (like sperm and eggs) are called g_____.</v>
       </c>
     </row>
     <row r="21">
@@ -1007,7 +1007,7 @@
         <v>Fertilisation which occurs outside the body of the parents</v>
       </c>
       <c r="I21" t="str">
-        <v>External fertilisation is when _____.</v>
+        <v>External fertilisation occurs o_____ the body of the parents.</v>
       </c>
     </row>
     <row r="22">
@@ -1036,7 +1036,7 @@
         <v>Fertilisation which occurs inside the body of the female</v>
       </c>
       <c r="I22" t="str">
-        <v>Internal fertilisation is when _____.</v>
+        <v>Internal fertilisation occurs i_____ the body of the female.</v>
       </c>
     </row>
     <row r="23">
@@ -1065,7 +1065,7 @@
         <v>Testis, sperm duct, penis</v>
       </c>
       <c r="I23" t="str">
-        <v>The 3 key parts of the male reproductive system are _____.</v>
+        <v>The 3 key parts of the male reproductive system: the t_____, s_____ d_____ and p_____.</v>
       </c>
     </row>
     <row r="24">
@@ -1094,7 +1094,7 @@
         <v>Ovary, fallopian tubes, cervix, uterus, vagina</v>
       </c>
       <c r="I24" t="str">
-        <v>The 5 key parts of the female reproductive system are _____.</v>
+        <v>The 5 key parts of the female reproductive system: o_____, f_____ t_____, c_____, u_____ and v_____.</v>
       </c>
     </row>
     <row r="25">
@@ -1123,7 +1123,7 @@
         <v>A time when a woman's ovaries stop releasing egg cells</v>
       </c>
       <c r="I25" t="str">
-        <v>Menopause is _____.</v>
+        <v>The time when a woman's ovaries stop releasing egg cells is called m_____.</v>
       </c>
     </row>
     <row r="26">
@@ -1152,7 +1152,7 @@
         <v>The testes</v>
       </c>
       <c r="I26" t="str">
-        <v>Sperm cells are made in _____.</v>
+        <v>Sperm cells are made in the t_____.</v>
       </c>
     </row>
     <row r="27">
@@ -1181,7 +1181,7 @@
         <v>oxygen and nutrients (or named nutrient)</v>
       </c>
       <c r="I27" t="str">
-        <v>Two substances that pass from the baby to the mother's blood via the placenta are _____.</v>
+        <v>Two substances that pass from the baby to the mother's blood via the placenta: o_____ and n_____.</v>
       </c>
     </row>
     <row r="28">
@@ -1210,7 +1210,7 @@
         <v>Carbon dioxide and waste products (or urea)</v>
       </c>
       <c r="I28" t="str">
-        <v>Two substances that pass from the mother's blood to the baby via the placenta are _____.</v>
+        <v>Two substances that pass from the mother's blood to the baby via the placenta: c_____ d_____ and w_____ p_____.</v>
       </c>
     </row>
     <row r="29">
@@ -1239,7 +1239,7 @@
         <v>To protect the baby</v>
       </c>
       <c r="I29" t="str">
-        <v>The role of amniotic fluid is _____.</v>
+        <v>The role of amniotic fluid is to p_____ the developing baby.</v>
       </c>
     </row>
     <row r="30">
@@ -1268,7 +1268,7 @@
         <v>9 months</v>
       </c>
       <c r="I30" t="str">
-        <v>Human pregnancy lasts approximately _____.</v>
+        <v>Human pregnancy lasts approximately _____ months.</v>
       </c>
     </row>
     <row r="31">
@@ -1297,7 +1297,7 @@
         <v>Time take for a baby to develop from fertilisation</v>
       </c>
       <c r="I31" t="str">
-        <v>The gestation period is _____.</v>
+        <v>The time taken for a baby to develop from fertilisation to birth is called the g_____ p_____.</v>
       </c>
     </row>
     <row r="32">
@@ -1326,7 +1326,7 @@
         <v>Organ providing foetus with oxygen and nutrients</v>
       </c>
       <c r="I32" t="str">
-        <v>The placenta is _____.</v>
+        <v>The organ that provides the foetus with oxygen and nutrients is called the p_____.</v>
       </c>
     </row>
     <row r="33">
@@ -1355,7 +1355,7 @@
         <v>Tube connecting foetus to placenta</v>
       </c>
       <c r="I33" t="str">
-        <v>The umbilical cord is _____.</v>
+        <v>The tube that connects the foetus to the placenta is called the u_____ c_____.</v>
       </c>
     </row>
     <row r="34">
@@ -1384,7 +1384,7 @@
         <v>Losing uterus lining</v>
       </c>
       <c r="I34" t="str">
-        <v>Menstruation is _____.</v>
+        <v>The monthly shedding of the uterus lining is called m_____.</v>
       </c>
     </row>
     <row r="35">
@@ -1413,7 +1413,7 @@
         <v>Releasing an egg</v>
       </c>
       <c r="I35" t="str">
-        <v>Ovulation is _____.</v>
+        <v>The release of an egg from the ovary is called o_____.</v>
       </c>
     </row>
     <row r="36">
@@ -1442,7 +1442,7 @@
         <v>FSH (follicle stimulating hormone)</v>
       </c>
       <c r="I36" t="str">
-        <v>The hormone that causes egg maturation in the ovaries is _____.</v>
+        <v>The hormone that causes egg maturation in the ovaries is F_____ (follicle stimulating hormone).</v>
       </c>
     </row>
     <row r="37">
@@ -1471,7 +1471,7 @@
         <v>Progesterone</v>
       </c>
       <c r="I37" t="str">
-        <v>The hormone that maintains the uterus lining is _____.</v>
+        <v>The hormone that maintains the uterus lining is p_____.</v>
       </c>
     </row>
     <row r="38">
@@ -1500,7 +1500,7 @@
         <v>Contracts and flattens</v>
       </c>
       <c r="I38" t="str">
-        <v>When we breathe in, the diaphragm _____.</v>
+        <v>When we breathe in, the diaphragm c_____ and f_____.</v>
       </c>
     </row>
     <row r="39">
@@ -1529,7 +1529,7 @@
         <v>Relaxes and return to dome shape</v>
       </c>
       <c r="I39" t="str">
-        <v>When we breathe out, the diaphragm _____.</v>
+        <v>When we breathe out, the diaphragm r_____ and returns to a d_____ shape.</v>
       </c>
     </row>
     <row r="40">
@@ -1558,7 +1558,7 @@
         <v>Arteries, veins and capillaries</v>
       </c>
       <c r="I40" t="str">
-        <v>The three types of blood vessel are _____.</v>
+        <v>The three types of blood vessel are a_____, v_____ and c_____.</v>
       </c>
     </row>
     <row r="41">
@@ -1587,7 +1587,7 @@
         <v>Protect the heart and lungs</v>
       </c>
       <c r="I41" t="str">
-        <v>The function of the ribcage is to _____.</v>
+        <v>The function of the ribcage is to p_____ the heart and lungs.</v>
       </c>
     </row>
     <row r="42">
@@ -1616,7 +1616,7 @@
         <v>To protect against infection</v>
       </c>
       <c r="I42" t="str">
-        <v>The purpose of white blood cells is _____.</v>
+        <v>The purpose of white blood cells is to p_____ the body against i_____.</v>
       </c>
     </row>
     <row r="43">
@@ -1645,7 +1645,7 @@
         <v>Bone marrow</v>
       </c>
       <c r="I43" t="str">
-        <v>Blood cells are made in _____.</v>
+        <v>Blood cells are made in the b_____ m_____.</v>
       </c>
     </row>
     <row r="44">
@@ -1674,7 +1674,7 @@
         <v>1. Support2. protect vital organs 3. movement 4. make blood cells</v>
       </c>
       <c r="I44" t="str">
-        <v>The 4 main functions of the skeleton are _____.</v>
+        <v>The 4 main functions of the skeleton: s_____, p_____ vital organs, e_____ m_____ and making b_____ c_____.</v>
       </c>
     </row>
     <row r="45">
@@ -1703,7 +1703,7 @@
         <v>cartilage</v>
       </c>
       <c r="I45" t="str">
-        <v>The smooth substance found at the end of a bone is _____.</v>
+        <v>The smooth substance found at the end of bones is called c_____.</v>
       </c>
     </row>
     <row r="46">
@@ -1732,7 +1732,7 @@
         <v>Ball and socket</v>
       </c>
       <c r="I46" t="str">
-        <v>A hip joint is a _____ joint.</v>
+        <v>A hip joint is an example of a b_____ and s_____ joint.</v>
       </c>
     </row>
     <row r="47">
@@ -1761,7 +1761,7 @@
         <v>calcium</v>
       </c>
       <c r="I47" t="str">
-        <v>The mineral that makes bones strong is _____.</v>
+        <v>The mineral that makes bones strong is c_____.</v>
       </c>
     </row>
     <row r="48">
@@ -1790,7 +1790,7 @@
         <v>quadriceps and hamstrings</v>
       </c>
       <c r="I48" t="str">
-        <v>An example of a pair of antagonistic muscles in the legs is _____.</v>
+        <v>An example of antagonistic muscles in the legs: the q_____ and h_____.</v>
       </c>
     </row>
     <row r="49">
@@ -1819,7 +1819,7 @@
         <v>Joints</v>
       </c>
       <c r="I49" t="str">
-        <v>Bones are linked together by _____.</v>
+        <v>Bones are linked together at j_____.</v>
       </c>
     </row>
     <row r="50">
@@ -1848,7 +1848,7 @@
         <v>By strong tendons</v>
       </c>
       <c r="I50" t="str">
-        <v>Muscles are attached to bone by _____.</v>
+        <v>Muscles are attached to bone by strong t_____.</v>
       </c>
     </row>
     <row r="51">
@@ -1877,7 +1877,7 @@
         <v>By getting shorter - contraction</v>
       </c>
       <c r="I51" t="str">
-        <v>Muscles work by _____.</v>
+        <v>Muscles work by getting shorter — a process called c_____.</v>
       </c>
     </row>
     <row r="52">
@@ -1906,7 +1906,7 @@
         <v>Alcohol</v>
       </c>
       <c r="I52" t="str">
-        <v>An example of a depressant drug is _____.</v>
+        <v>An example of a d_____ drug (one that slows the nervous system) is alcohol.</v>
       </c>
     </row>
     <row r="53">
@@ -1935,7 +1935,7 @@
         <v>MDMA, Marijuana</v>
       </c>
       <c r="I53" t="str">
-        <v>An example of a hallucinogen is _____.</v>
+        <v>An example of a h_____ (a drug that causes hallucinations) is MDMA or marijuana.</v>
       </c>
     </row>
     <row r="54">
@@ -1964,7 +1964,7 @@
         <v>Ibuprofen, Morphone</v>
       </c>
       <c r="I54" t="str">
-        <v>An example of a painkiller is _____.</v>
+        <v>An example of a p_____ drug is ibuprofen or morphine.</v>
       </c>
     </row>
     <row r="55">
@@ -1993,7 +1993,7 @@
         <v>Tobacco, Caffeine</v>
       </c>
       <c r="I55" t="str">
-        <v>An example of a stimulant is _____.</v>
+        <v>An example of a s_____ drug (one that speeds the nervous system) is caffeine or tobacco.</v>
       </c>
     </row>
     <row r="56">
@@ -2022,7 +2022,7 @@
         <v>The environment that an organism lives in</v>
       </c>
       <c r="I56" t="str">
-        <v>A habitat is _____.</v>
+        <v>The environment that an organism lives in is called its h_____.</v>
       </c>
     </row>
     <row r="57">
@@ -2051,7 +2051,7 @@
         <v>Any sensible answer</v>
       </c>
       <c r="I57" t="str">
-        <v>Two examples of continuous variation in humans are _____.</v>
+        <v>Two examples of c_____ variation in humans are height and weight.</v>
       </c>
     </row>
     <row r="58">
@@ -2080,7 +2080,7 @@
         <v>Any sensible answer</v>
       </c>
       <c r="I58" t="str">
-        <v>Two examples of discontinuous variation in humans are _____.</v>
+        <v>Two examples of d_____ variation in humans are blood type and eye colour.</v>
       </c>
     </row>
     <row r="59">
@@ -2109,7 +2109,7 @@
         <v>The living and non-living things in a given area</v>
       </c>
       <c r="I59" t="str">
-        <v>An ecosystem is _____.</v>
+        <v>All the living and non-living things in a given area make up an e_____.</v>
       </c>
     </row>
     <row r="60">
@@ -2138,7 +2138,7 @@
         <v>Organisms that have similar characteristics and can reproduce to produce FERTILE offspring</v>
       </c>
       <c r="I60" t="str">
-        <v>A species is _____.</v>
+        <v>Organisms that can interbreed to produce fertile offspring belong to the same s_____.</v>
       </c>
     </row>
     <row r="61">
@@ -2167,7 +2167,7 @@
         <v>Characteristics inherited from your parents. Any reasonable examples</v>
       </c>
       <c r="I61" t="str">
-        <v>Inherited variation refers to _____.</v>
+        <v>Inherited variation refers to c_____ passed on from your p_____, such as eye colour.</v>
       </c>
     </row>
     <row r="62">
@@ -2196,7 +2196,7 @@
         <v>Camouflage, pointy teeth and claws, forward facing eyes, any other reasonable answer</v>
       </c>
       <c r="I62" t="str">
-        <v>Three adaptations that help a tiger survive in its environment include _____.</v>
+        <v>Three adaptations that help a tiger survive: c_____, sharp t_____ and c_____, and f_____-facing eyes.</v>
       </c>
     </row>
     <row r="63">
@@ -2225,7 +2225,7 @@
         <v>hibernation, shedding winter coat, migration, etc.</v>
       </c>
       <c r="I63" t="str">
-        <v>Two adaptations animals show in response to seasonal changes include _____.</v>
+        <v>Two seasonal adaptations in animals include h_____ and m_____.</v>
       </c>
     </row>
     <row r="64">
@@ -2254,7 +2254,7 @@
         <v>They hibernate</v>
       </c>
       <c r="I64" t="str">
-        <v>Hedgehogs survive winter by _____.</v>
+        <v>Hedgehogs survive winter by h_____.</v>
       </c>
     </row>
     <row r="65">
@@ -2283,7 +2283,7 @@
         <v>To reduce water loss and nutrient expenditure</v>
       </c>
       <c r="I65" t="str">
-        <v>Deciduous trees lose their leaves in winter to _____.</v>
+        <v>Deciduous trees lose their leaves in winter to reduce w_____ l_____ and save energy.</v>
       </c>
     </row>
     <row r="66">
@@ -2312,7 +2312,7 @@
         <v>An organism that eats only other animals</v>
       </c>
       <c r="I66" t="str">
-        <v>A carnivore is _____.</v>
+        <v>An organism that only eats other animals is called a c_____.</v>
       </c>
     </row>
     <row r="67">
@@ -2341,7 +2341,7 @@
         <v>Organisms trying to gain a share of limited resources</v>
       </c>
       <c r="I67" t="str">
-        <v>Competition is _____.</v>
+        <v>When organisms fight for a share of limited resources, this is called c_____.</v>
       </c>
     </row>
     <row r="68">
@@ -2370,7 +2370,7 @@
         <v>An organism that eats another organism</v>
       </c>
       <c r="I68" t="str">
-        <v>A consumer is _____.</v>
+        <v>An organism that feeds on other organisms is called a c_____.</v>
       </c>
     </row>
     <row r="69">
@@ -2399,7 +2399,7 @@
         <v>Organisms that break down dead plant and animal material</v>
       </c>
       <c r="I69" t="str">
-        <v>A decomposer is _____.</v>
+        <v>Organisms that break down dead material and return nutrients to the soil are called d_____.</v>
       </c>
     </row>
     <row r="70">
@@ -2428,7 +2428,7 @@
         <v>Chemicals (in particular toxins) concentrate in the bodies of consumers the further along the food chain they are, potentially leading to fatal levels</v>
       </c>
       <c r="I70" t="str">
-        <v>Bioaccumulation is when _____.</v>
+        <v>The process where toxins build up to higher concentrations further along a food chain is called b_____.</v>
       </c>
     </row>
     <row r="71">
@@ -2457,7 +2457,7 @@
         <v>Correct shaped pyramid labelled</v>
       </c>
       <c r="I71" t="str">
-        <v>In a pyramid of biomass for the chain rose bush → aphids → ladybirds, the _____ forms the widest bar at the base.</v>
+        <v>In a pyramid of biomass, the producer (e.g. r_____ b_____) always forms the widest bar at the base.</v>
       </c>
     </row>
     <row r="72">
@@ -2486,7 +2486,7 @@
         <v>Correct shaped pyramid labelled</v>
       </c>
       <c r="I72" t="str">
-        <v>In the food chain grass → grasshopper → frog → snake, the pyramid of numbers has _____ at the base with the widest bar.</v>
+        <v>In a pyramid of numbers for grass → grasshopper → frog → snake, the bar for g_____ is widest at the base.</v>
       </c>
     </row>
     <row r="73">
@@ -2515,7 +2515,7 @@
         <v>A substance made of a single element or compound</v>
       </c>
       <c r="I73" t="str">
-        <v>In chemistry, a pure substance is _____.</v>
+        <v>In chemistry, a substance made of only one element or compound is called p_____.</v>
       </c>
     </row>
     <row r="74">
@@ -2544,7 +2544,7 @@
         <v>A substance that has had nothing added to it and is in its "natural" state</v>
       </c>
       <c r="I74" t="str">
-        <v>In everyday language, a pure substance is _____.</v>
+        <v>In everyday language, a pure substance is one that has had n_____ added to it.</v>
       </c>
     </row>
     <row r="75">
@@ -2573,7 +2573,7 @@
         <v>1) filter funnel, 2) filter paper</v>
       </c>
       <c r="I75" t="str">
-        <v>The two pieces of equipment needed for filtration are _____.</v>
+        <v>The two pieces of equipment needed for filtration: a f_____ f_____ and f_____ p_____.</v>
       </c>
     </row>
     <row r="76">
@@ -2602,7 +2602,7 @@
         <v>Filtration</v>
       </c>
       <c r="I76" t="str">
-        <v>To separate an insoluble solute from solution we use _____.</v>
+        <v>To separate an insoluble solid from a liquid we use f_____.</v>
       </c>
     </row>
     <row r="77">
@@ -2631,7 +2631,7 @@
         <v>Stir and heat</v>
       </c>
       <c r="I77" t="str">
-        <v>Three ways of increasing the rate of dissolving include _____.</v>
+        <v>Three ways to speed up dissolving: s_____, h_____ and grinding into smaller pieces.</v>
       </c>
     </row>
     <row r="78">
@@ -2660,7 +2660,7 @@
         <v>Soluble</v>
       </c>
       <c r="I78" t="str">
-        <v>Salt is _____ in water.</v>
+        <v>Salt is s_____ in water.</v>
       </c>
     </row>
     <row r="79">
@@ -2689,7 +2689,7 @@
         <v>Insoluble</v>
       </c>
       <c r="I79" t="str">
-        <v>Sand is _____ in water.</v>
+        <v>Sand is i_____ in water.</v>
       </c>
     </row>
     <row r="80">
@@ -2718,7 +2718,7 @@
         <v>Soluble</v>
       </c>
       <c r="I80" t="str">
-        <v>Sugar is _____ in water.</v>
+        <v>Sugar is s_____ in water.</v>
       </c>
     </row>
     <row r="81">
@@ -2747,7 +2747,7 @@
         <v>Evaporation</v>
       </c>
       <c r="I81" t="str">
-        <v>To separate a soluble solute from solution we use _____.</v>
+        <v>To separate a dissolved solid from a solution we use e_____.</v>
       </c>
     </row>
     <row r="82">
@@ -2776,7 +2776,7 @@
         <v>100 degrees Celsius</v>
       </c>
       <c r="I82" t="str">
-        <v>The boiling point of water is _____.</v>
+        <v>The boiling point of water is _____ °C.</v>
       </c>
     </row>
     <row r="83">
@@ -2805,7 +2805,7 @@
         <v>Evaporation can happen at ay temperature, boiling only happens at the boiling point of a substance.</v>
       </c>
       <c r="I83" t="str">
-        <v>Unlike boiling, evaporation _____.</v>
+        <v>Unlike boiling, evaporation can occur at a_____ t_____.</v>
       </c>
     </row>
     <row r="84">
@@ -2834,7 +2834,7 @@
         <v>Line drawn with a pen, solvent level above the ink being separated</v>
       </c>
       <c r="I84" t="str">
-        <v>Two errors that can occur when carrying out chromatography are _____.</v>
+        <v>Two errors in chromatography: drawing the start line with a p_____, and solvent level being a_____ the sample line.</v>
       </c>
     </row>
     <row r="85">
@@ -2863,7 +2863,7 @@
         <v>Chromatography</v>
       </c>
       <c r="I85" t="str">
-        <v>To separate two or more coloured solutions we use _____.</v>
+        <v>To separate a mixture of coloured dyes we use c_____.</v>
       </c>
     </row>
     <row r="86">
@@ -2892,7 +2892,7 @@
         <v>To prevent it from dissolving in the solvent and affecting our results.</v>
       </c>
       <c r="I86" t="str">
-        <v>The starting line on a chromatogram is drawn in pencil because _____.</v>
+        <v>The start line on a chromatogram is drawn in p_____ so it doesn't d_____ in the solvent.</v>
       </c>
     </row>
     <row r="87">
@@ -2921,7 +2921,7 @@
         <v>1) evaporating basin, 2) tripod, 3) gauze, 4) heat proof mat, 5) Bunsen burner</v>
       </c>
       <c r="I87" t="str">
-        <v>The five pieces of equipment needed for evaporation are _____.</v>
+        <v>The 5 pieces of equipment for evaporation: e_____ b_____, t_____, g_____, h_____ p_____ m_____ and B_____ b_____.</v>
       </c>
     </row>
     <row r="88">
@@ -2950,7 +2950,7 @@
         <v>Heat (evaporate liquid) and then cool (condense)</v>
       </c>
       <c r="I88" t="str">
-        <v>The two stages of distillation are _____.</v>
+        <v>Distillation has two stages: first h_____ to evaporate the liquid, then c_____ to condense the vapour.</v>
       </c>
     </row>
     <row r="89">
@@ -2979,7 +2979,7 @@
         <v>Distillation</v>
       </c>
       <c r="I89" t="str">
-        <v>To separate a solvent from solution we use _____.</v>
+        <v>To separate a solvent from a solution we use d_____.</v>
       </c>
     </row>
     <row r="90">
@@ -3008,7 +3008,7 @@
         <v>Correct symbol drawn</v>
       </c>
       <c r="I90" t="str">
-        <v>The hazard symbol for a flammable substance shows _____.</v>
+        <v>The hazard symbol for flammable substances shows a f_____.</v>
       </c>
     </row>
     <row r="91">
@@ -3037,7 +3037,7 @@
         <v>The substance reacts with metals and organic materials, wearing away or corroding them.</v>
       </c>
       <c r="I91" t="str">
-        <v>A corrosive substance is one that _____.</v>
+        <v>A c_____ substance reacts with metals and organic materials, wearing them away.</v>
       </c>
     </row>
     <row r="92">
@@ -3066,7 +3066,7 @@
         <v>Irritant/harmful</v>
       </c>
       <c r="I92" t="str">
-        <v>The exclamation mark hazard symbol represents _____.</v>
+        <v>The exclamation mark hazard symbol represents something i_____ or h_____.</v>
       </c>
     </row>
     <row r="93">
@@ -3095,7 +3095,7 @@
         <v>Litmus paper and universal indicator</v>
       </c>
       <c r="I93" t="str">
-        <v>Two examples of indicators are _____.</v>
+        <v>Two examples of indicators are l_____ paper and u_____ i_____.</v>
       </c>
     </row>
     <row r="94">
@@ -3124,7 +3124,7 @@
         <v>Red</v>
       </c>
       <c r="I94" t="str">
-        <v>Universal indicator turns _____ in a strong acid.</v>
+        <v>Universal indicator turns r_____ in a strong acid.</v>
       </c>
     </row>
     <row r="95">
@@ -3153,7 +3153,7 @@
         <v>Orange</v>
       </c>
       <c r="I95" t="str">
-        <v>Universal indicator turns _____ in a weak acid.</v>
+        <v>Universal indicator turns o_____ in a weak acid.</v>
       </c>
     </row>
     <row r="96">
@@ -3182,7 +3182,7 @@
         <v>Indicator</v>
       </c>
       <c r="I96" t="str">
-        <v>A substance that changes colour in acid or alkali is called an _____.</v>
+        <v>A substance that changes colour in acid or alkali is called an i_____.</v>
       </c>
     </row>
     <row r="97">
@@ -3211,7 +3211,7 @@
         <v>Purple</v>
       </c>
       <c r="I97" t="str">
-        <v>Universal indicator turns _____ in an alkali.</v>
+        <v>Universal indicator turns p_____ in an alkali.</v>
       </c>
     </row>
     <row r="98">
@@ -3240,7 +3240,7 @@
         <v>Green</v>
       </c>
       <c r="I98" t="str">
-        <v>Universal indicator turns _____ in a neutral substance.</v>
+        <v>Universal indicator turns g_____ in a neutral substance.</v>
       </c>
     </row>
     <row r="99">
@@ -3298,7 +3298,7 @@
         <v>pH 1-3</v>
       </c>
       <c r="I100" t="str">
-        <v>A strong acid has a pH of _____.</v>
+        <v>A strong acid has a pH of between _____ and _____.</v>
       </c>
     </row>
     <row r="101">
@@ -3327,7 +3327,7 @@
         <v>The reaction of an acid with an alkali to form a neutral salt and water</v>
       </c>
       <c r="I101" t="str">
-        <v>Neutralisation is _____.</v>
+        <v>The reaction between an acid and an alkali to form a salt and water is called n_____.</v>
       </c>
     </row>
     <row r="102">
@@ -3356,7 +3356,7 @@
         <v>Acid + alkali -&gt; salt + water</v>
       </c>
       <c r="I102" t="str">
-        <v>The general equation for a neutralisation reaction is _____.</v>
+        <v>The general equation for neutralisation is: a_____ + a_____ → s_____ + w_____.</v>
       </c>
     </row>
     <row r="103">
@@ -3443,7 +3443,7 @@
         <v>Magnesium chloride and water</v>
       </c>
       <c r="I105" t="str">
-        <v>When magnesium hydroxide reacts with hydrochloric acid, the two products formed are _____.</v>
+        <v>When magnesium hydroxide reacts with hydrochloric acid, the products are m_____ c_____ and w_____.</v>
       </c>
     </row>
     <row r="106">
@@ -3472,7 +3472,7 @@
         <v>Alkaline</v>
       </c>
       <c r="I106" t="str">
-        <v>Bleach is _____ (acidic or alkaline).</v>
+        <v>Bleach is a_____ — it has a pH above 7.</v>
       </c>
     </row>
     <row r="107">
@@ -3501,7 +3501,7 @@
         <v>Alkaline</v>
       </c>
       <c r="I107" t="str">
-        <v>Toothpaste is _____ (acidic or alkaline).</v>
+        <v>Toothpaste is a_____ — it has a pH above 7.</v>
       </c>
     </row>
     <row r="108">
@@ -3530,7 +3530,7 @@
         <v>Volume</v>
       </c>
       <c r="I108" t="str">
-        <v>The property measured in metres cubed (m³) is _____.</v>
+        <v>The property measured in metres cubed (m³) is v_____.</v>
       </c>
     </row>
     <row r="109">
@@ -3559,7 +3559,7 @@
         <v>Gases only.</v>
       </c>
       <c r="I109" t="str">
-        <v>Of the three states of matter, only _____ can be compressed.</v>
+        <v>Of the three states of matter, only g_____ can be compressed.</v>
       </c>
     </row>
     <row r="110">
@@ -3588,7 +3588,7 @@
         <v>Liquids and gases</v>
       </c>
       <c r="I110" t="str">
-        <v>The states of matter that can flow are _____.</v>
+        <v>The two states of matter that can flow are l_____ and g_____.</v>
       </c>
     </row>
     <row r="111">
@@ -3617,7 +3617,7 @@
         <v>The temperature at which a liquid turns into a gas</v>
       </c>
       <c r="I111" t="str">
-        <v>The boiling point is _____.</v>
+        <v>The temperature at which a liquid turns into a gas is called the b_____ p_____.</v>
       </c>
     </row>
     <row r="112">
@@ -3646,7 +3646,7 @@
         <v>Quick and random</v>
       </c>
       <c r="I112" t="str">
-        <v>Particles in a gas move _____.</v>
+        <v>Particles in a gas move q_____ and r_____.</v>
       </c>
     </row>
     <row r="113">
@@ -3675,7 +3675,7 @@
         <v>Slide over each other</v>
       </c>
       <c r="I113" t="str">
-        <v>Particles in a liquid _____.</v>
+        <v>Particles in a liquid can s_____ over each other.</v>
       </c>
     </row>
     <row r="114">
@@ -3704,7 +3704,7 @@
         <v>Vibrate</v>
       </c>
       <c r="I114" t="str">
-        <v>Particles in a solid _____.</v>
+        <v>Particles in a solid only v_____ on the spot.</v>
       </c>
     </row>
     <row r="115">
@@ -3733,7 +3733,7 @@
         <v>The random movement of particles in a fluid</v>
       </c>
       <c r="I115" t="str">
-        <v>Brownian motion is _____.</v>
+        <v>The random movement of microscopic particles in a fluid is called B_____ m_____.</v>
       </c>
     </row>
     <row r="116">
@@ -3762,7 +3762,7 @@
         <v>1,000,000,000nm</v>
       </c>
       <c r="I116" t="str">
-        <v>There are _____ nanometres in one metre.</v>
+        <v>There are 1,000,000,000 n_____ in one metre.</v>
       </c>
     </row>
     <row r="117">
@@ -3791,7 +3791,7 @@
         <v>Liquids and gases</v>
       </c>
       <c r="I117" t="str">
-        <v>Brownian motion occurs in _____.</v>
+        <v>Brownian motion occurs in l_____ and g_____.</v>
       </c>
     </row>
     <row r="118">
@@ -3820,7 +3820,7 @@
         <v>The movement of particles from a low concentration to a high concentration using energy</v>
       </c>
       <c r="I118" t="str">
-        <v>Active transport is _____.</v>
+        <v>The movement of particles from low to high concentration using energy is called a_____ t_____.</v>
       </c>
     </row>
     <row r="119">
@@ -3849,7 +3849,7 @@
         <v>The movement of particles from a high concentration to a low concentration</v>
       </c>
       <c r="I119" t="str">
-        <v>Diffusion is _____.</v>
+        <v>The movement of particles from high to low concentration is called d_____.</v>
       </c>
     </row>
     <row r="120">
@@ -3878,7 +3878,7 @@
         <v>The movement of water particles from a dilute to a concentrated solution through a partially permeable membrane</v>
       </c>
       <c r="I120" t="str">
-        <v>Osmosis is _____.</v>
+        <v>The movement of water through a partially permeable membrane from a dilute to concentrated solution is called o_____.</v>
       </c>
     </row>
     <row r="121">
@@ -3907,7 +3907,7 @@
         <v>Solid</v>
       </c>
       <c r="I121" t="str">
-        <v>Diffusion does not occur in _____.</v>
+        <v>Diffusion does not occur in a s_____.</v>
       </c>
     </row>
     <row r="122">
@@ -3936,7 +3936,7 @@
         <v>Pressure increases</v>
       </c>
       <c r="I122" t="str">
-        <v>When a gas is heated, its pressure _____.</v>
+        <v>When a gas is heated, its pressure i_____.</v>
       </c>
     </row>
     <row r="123">
@@ -3965,7 +3965,7 @@
         <v>There are more particles of air in the same volume, which leads to more collisions with the walls of the tyre, causing a higher pressure.</v>
       </c>
       <c r="I123" t="str">
-        <v>Pumping up a tyre increases air pressure because _____.</v>
+        <v>Pumping air into a tyre increases pressure because there are more p_____ causing more c_____ with the walls.</v>
       </c>
     </row>
     <row r="124">
@@ -3994,7 +3994,7 @@
         <v>The pressure in the straw is less than the pressure on the surface of your drink, pushing the drink up the straw.</v>
       </c>
       <c r="I124" t="str">
-        <v>Sucking on a straw draws liquid upward because _____.</v>
+        <v>Sucking on a straw lowers p_____ inside it, so higher pressure outside p_____ the liquid up.</v>
       </c>
     </row>
     <row r="125">
@@ -4023,7 +4023,7 @@
         <v>Tiny particles</v>
       </c>
       <c r="I125" t="str">
-        <v>An atom is _____.</v>
+        <v>The tiny building blocks that make up all matter are called a_____.</v>
       </c>
     </row>
     <row r="126">
@@ -4052,7 +4052,7 @@
         <v>A group of atoms bonded together</v>
       </c>
       <c r="I126" t="str">
-        <v>A molecule is _____.</v>
+        <v>A group of atoms chemically bonded together is called a m_____.</v>
       </c>
     </row>
     <row r="127">
@@ -4081,7 +4081,7 @@
         <v>Elements</v>
       </c>
       <c r="I127" t="str">
-        <v>Substances made of only one type of atom are called _____.</v>
+        <v>Substances made of only one type of atom are called e_____.</v>
       </c>
     </row>
     <row r="128">
@@ -4110,7 +4110,7 @@
         <v>Compounds</v>
       </c>
       <c r="I128" t="str">
-        <v>Substances made of two or more types of atoms chemically bonded together are called _____.</v>
+        <v>Substances made of two or more types of atoms chemically bonded together are called c_____.</v>
       </c>
     </row>
     <row r="129">
@@ -4255,7 +4255,7 @@
         <v>Iron, nickel and cobalt.</v>
       </c>
       <c r="I133" t="str">
-        <v>Three magnetic elements are _____.</v>
+        <v>Three magnetic elements are i_____, n_____ and c_____.</v>
       </c>
     </row>
     <row r="134">
@@ -4284,7 +4284,7 @@
         <v>Solids with high melting points, strong, flexible, malleable, shiny  when polished, good conductor of heat, good conductor of electricity</v>
       </c>
       <c r="I134" t="str">
-        <v>Four properties of most metals include _____.</v>
+        <v>Four properties of most metals: h_____ m_____ point, good c_____ of heat and electricity, d_____ and m_____.</v>
       </c>
     </row>
     <row r="135">
@@ -4313,7 +4313,7 @@
         <v>Low melting points, brittle when solid, not shiny, poor conductor of heat, poor conductor of electricity.</v>
       </c>
       <c r="I135" t="str">
-        <v>Four properties of most non-metals include _____.</v>
+        <v>Four properties of most non-metals: l_____ m_____ point, b_____ when solid, not s_____, poor c_____.</v>
       </c>
     </row>
     <row r="136">
@@ -4342,7 +4342,7 @@
         <v>Copper chloride</v>
       </c>
       <c r="I136" t="str">
-        <v>When chlorine gas reacts with copper, _____ is formed.</v>
+        <v>When chlorine gas reacts with copper, c_____ c_____ is formed.</v>
       </c>
     </row>
     <row r="137">
@@ -4371,7 +4371,7 @@
         <v>-ide</v>
       </c>
       <c r="I137" t="str">
-        <v>Substances made of a metal and non-metal chemically bonded together usually end in _____.</v>
+        <v>Substances made of a metal and non-metal chemically bonded together usually end in _____-ide.</v>
       </c>
     </row>
     <row r="138">
@@ -4400,7 +4400,7 @@
         <v>A reaction that gives out heat</v>
       </c>
       <c r="I138" t="str">
-        <v>An exothermic reaction is one that _____.</v>
+        <v>A reaction that releases heat energy to the surroundings is called e_____.</v>
       </c>
     </row>
     <row r="139">
@@ -4429,7 +4429,7 @@
         <v>Colour change, change in temperature, fizzing, combustion, smell, a gas being given off, a solid forming.</v>
       </c>
       <c r="I139" t="str">
-        <v>Three signs that a chemical reaction may have occurred include _____.</v>
+        <v>Three signs of a chemical reaction: c_____ change, change in t_____ and f_____.</v>
       </c>
     </row>
     <row r="140">
@@ -4458,7 +4458,7 @@
         <v>-ate</v>
       </c>
       <c r="I140" t="str">
-        <v>Substances made of a metal, a non-metal and oxygen chemically bonded together usually end in _____.</v>
+        <v>Substances made of a metal, a non-metal and oxygen chemically bonded together usually end in _____-ate.</v>
       </c>
     </row>
     <row r="141">
@@ -4487,7 +4487,7 @@
         <v>When heat is used to break down a reactant into two or more products.</v>
       </c>
       <c r="I141" t="str">
-        <v>A thermal decomposition reaction is when _____.</v>
+        <v>A reaction in which h_____ is used to break down one substance into two or more products is called t_____ d_____.</v>
       </c>
     </row>
     <row r="142">
@@ -4516,7 +4516,7 @@
         <v>Amount of energy (in food) available</v>
       </c>
       <c r="I142" t="str">
-        <v>A calorie is _____.</v>
+        <v>The unit used to measure the amount of energy available in food is called a c_____.</v>
       </c>
     </row>
     <row r="143">
@@ -4545,7 +4545,7 @@
         <v>Joule (J)</v>
       </c>
       <c r="I143" t="str">
-        <v>The unit for energy is _____.</v>
+        <v>The standard unit for energy is the J_____.</v>
       </c>
     </row>
     <row r="144">
@@ -4574,7 +4574,7 @@
         <v>Combustion or respiration</v>
       </c>
       <c r="I144" t="str">
-        <v>The energy stored in food is released by _____.</v>
+        <v>The energy stored in food is released by c_____ or r_____.</v>
       </c>
     </row>
     <row r="145">
@@ -4603,7 +4603,7 @@
         <v>A lot of energy is available from most foods</v>
       </c>
       <c r="I145" t="str">
-        <v>Kilojoules are used on food labels because _____.</v>
+        <v>Kilojoules are used on food labels because the energy values in joules would be very l_____.</v>
       </c>
     </row>
     <row r="146">
@@ -4632,7 +4632,7 @@
         <v>Process of burning by heat</v>
       </c>
       <c r="I146" t="str">
-        <v>Combustion is _____.</v>
+        <v>The process of burning fuel to release heat and light energy is called c_____.</v>
       </c>
     </row>
     <row r="147">
@@ -4661,7 +4661,7 @@
         <v>Battery, Food</v>
       </c>
       <c r="I147" t="str">
-        <v>An example of a store of chemical energy is _____.</v>
+        <v>An example of a store of chemical energy is a b_____ or f_____.</v>
       </c>
     </row>
     <row r="148">
@@ -4690,7 +4690,7 @@
         <v>A chemical reaction which uses glucose and oxygen to release energy</v>
       </c>
       <c r="I148" t="str">
-        <v>Respiration is _____.</v>
+        <v>R_____ is the chemical reaction that uses glucose and oxygen to release energy in cells.</v>
       </c>
     </row>
     <row r="149">
@@ -4719,7 +4719,7 @@
         <v>three quarters</v>
       </c>
       <c r="I149" t="str">
-        <v>Approximately _____ of the UK's electricity is generated from fossil fuels.</v>
+        <v>Approximately t_____ q_____ of UK electricity is generated from fossil fuels.</v>
       </c>
     </row>
     <row r="150">
@@ -4748,7 +4748,7 @@
         <v>only used once and is in limited supply</v>
       </c>
       <c r="I150" t="str">
-        <v>A finite resource is one that _____.</v>
+        <v>A resource that is in limited supply and cannot be replaced is called a f_____ resource.</v>
       </c>
     </row>
     <row r="151">
@@ -4777,7 +4777,7 @@
         <v>cannot be replaced once they are all used up</v>
       </c>
       <c r="I151" t="str">
-        <v>A non-renewable energy resource is one that _____.</v>
+        <v>An energy resource that cannot be replaced once used up is called n_____-r_____.</v>
       </c>
     </row>
     <row r="152">
@@ -4806,7 +4806,7 @@
         <v>can be replaced, will not run out</v>
       </c>
       <c r="I152" t="str">
-        <v>A renewable energy source is one that _____.</v>
+        <v>An energy source that can be naturally replaced and will not run out is called r_____.</v>
       </c>
     </row>
     <row r="153">
@@ -4835,7 +4835,7 @@
         <v>Solar, wind, waves, hydroelectric, geothermal, biomass</v>
       </c>
       <c r="I153" t="str">
-        <v>Six examples of renewable energy resources are _____.</v>
+        <v>Six renewable energy resources: s_____, w_____, w_____, h_____, g_____ and b_____.</v>
       </c>
     </row>
     <row r="154">
@@ -4864,7 +4864,7 @@
         <v>The Sun</v>
       </c>
       <c r="I154" t="str">
-        <v>All the energy in our food originally comes from _____.</v>
+        <v>All the energy found in our food originally comes from the S_____.</v>
       </c>
     </row>
     <row r="155">
@@ -4893,7 +4893,7 @@
         <v>We can plant more of them</v>
       </c>
       <c r="I155" t="str">
-        <v>Biofuels can be considered renewable because _____.</v>
+        <v>Biofuels can be considered renewable because we can p_____ more of the source material.</v>
       </c>
     </row>
     <row r="156">
@@ -4922,7 +4922,7 @@
         <v>do not produce sulphur dioxide or carbon dioxide</v>
       </c>
       <c r="I156" t="str">
-        <v>An advantage of nuclear fuels is that they _____.</v>
+        <v>An advantage of nuclear fuels: they do not produce s_____ d_____ or c_____ d_____.</v>
       </c>
     </row>
     <row r="157">
@@ -4951,7 +4951,7 @@
         <v>non-renewable; if there is an accident radioactive material may be released into the environment, nuclear waste remains dangerous for thousands of years</v>
       </c>
       <c r="I157" t="str">
-        <v>Disadvantages of nuclear fuels include _____.</v>
+        <v>Disadvantages of nuclear fuels: n_____-r_____, r_____ waste and risk of accidents.</v>
       </c>
     </row>
     <row r="158">
@@ -4980,7 +4980,7 @@
         <v>Releases greenhouse gases, non-renewable</v>
       </c>
       <c r="I158" t="str">
-        <v>Two disadvantages of using fossil fuels to generate electricity are _____.</v>
+        <v>Two disadvantages of fossil fuels: they release g_____ g_____ and are n_____-r_____.</v>
       </c>
     </row>
     <row r="159">
@@ -5009,7 +5009,7 @@
         <v>Flow of electricity</v>
       </c>
       <c r="I159" t="str">
-        <v>Electric current is _____.</v>
+        <v>The flow of electric charge around a circuit is called c_____.</v>
       </c>
     </row>
     <row r="160">
@@ -5038,7 +5038,7 @@
         <v>Ampere (Amp)</v>
       </c>
       <c r="I160" t="str">
-        <v>The unit of electric current is _____.</v>
+        <v>The unit of electric current is the A_____ (amp).</v>
       </c>
     </row>
     <row r="161">
@@ -5067,7 +5067,7 @@
         <v>Ammeter</v>
       </c>
       <c r="I161" t="str">
-        <v>Electric current is measured using an _____.</v>
+        <v>Electric current is measured using an a_____.</v>
       </c>
     </row>
     <row r="162">
@@ -5096,7 +5096,7 @@
         <v>metal elements, graphite, mixtures of metal, salt solution, liquid calcium chloride</v>
       </c>
       <c r="I162" t="str">
-        <v>Examples of electrical conductors include _____.</v>
+        <v>Examples of electrical conductors include m_____, g_____ and s_____ s_____.</v>
       </c>
     </row>
     <row r="163">
@@ -5125,7 +5125,7 @@
         <v>most non-metal elements (e.g., sulphur, oxygen), diamond, plastic, wood, rock</v>
       </c>
       <c r="I163" t="str">
-        <v>Examples of electrical insulators include _____.</v>
+        <v>Examples of electrical insulators include p_____, w_____ and most n_____-m_____.</v>
       </c>
     </row>
     <row r="164">
@@ -5154,7 +5154,7 @@
         <v>set up a series circuit with a cell, lamp, wires &gt; place material in between two wires &gt; lamp on = conductor</v>
       </c>
       <c r="I164" t="str">
-        <v>To investigate how easily a material conducts electricity, you _____.</v>
+        <v>To test conductivity, set up a s_____ circuit with a lamp — if the lamp lights, the material is a c_____.</v>
       </c>
     </row>
     <row r="165">
@@ -5183,7 +5183,7 @@
         <v>a material that allows charge to move easily through it</v>
       </c>
       <c r="I165" t="str">
-        <v>An electrical conductor is _____.</v>
+        <v>A material that allows electric charge to move easily through it is called an electrical c_____.</v>
       </c>
     </row>
     <row r="166">
@@ -5212,7 +5212,7 @@
         <v>Components in a circuit are in separate loops</v>
       </c>
       <c r="I166" t="str">
-        <v>In a parallel circuit, _____.</v>
+        <v>A circuit where components are on separate branches is called a p_____ circuit.</v>
       </c>
     </row>
     <row r="167">
@@ -5241,7 +5241,7 @@
         <v>Components in a circuit are all in one loop</v>
       </c>
       <c r="I167" t="str">
-        <v>In a series circuit, _____.</v>
+        <v>A circuit where all components are connected in a single loop is called a s_____ circuit.</v>
       </c>
     </row>
     <row r="168">
@@ -5270,7 +5270,7 @@
         <v>The total current through the whole circuit is the sum of the currents through the separate components</v>
       </c>
       <c r="I168" t="str">
-        <v>In a parallel circuit, the total current is _____.</v>
+        <v>In a parallel circuit, the total current equals the s_____ of the currents in each branch.</v>
       </c>
     </row>
     <row r="169">
@@ -5299,7 +5299,7 @@
         <v>The current is the same at every point in the circuit and in every component</v>
       </c>
       <c r="I169" t="str">
-        <v>In a series circuit, the current is _____.</v>
+        <v>In a series circuit, the current is the s_____ at every point in the circuit.</v>
       </c>
     </row>
     <row r="170">
@@ -5328,7 +5328,7 @@
         <v>electrical conductor = low resistance, electrical insulator = high resistance</v>
       </c>
       <c r="I170" t="str">
-        <v>Compared to insulators, electrical conductors have _____ resistance.</v>
+        <v>Conductors have l_____ resistance; insulators have h_____ resistance.</v>
       </c>
     </row>
     <row r="171">
@@ -5357,7 +5357,7 @@
         <v>Energy carried by the flow of electrical charge</v>
       </c>
       <c r="I171" t="str">
-        <v>Potential difference (voltage) is _____.</v>
+        <v>The energy transferred per unit charge flowing around a circuit is called p_____ d_____ (or voltage).</v>
       </c>
     </row>
     <row r="172">
@@ -5386,7 +5386,7 @@
         <v>Slows down the flow of electricity</v>
       </c>
       <c r="I172" t="str">
-        <v>Resistance is _____.</v>
+        <v>The property that opposes and slows down the flow of electric current is called r_____.</v>
       </c>
     </row>
     <row r="173">
@@ -5415,7 +5415,7 @@
         <v>Volt (V)</v>
       </c>
       <c r="I173" t="str">
-        <v>The unit of potential difference is _____.</v>
+        <v>The unit of potential difference is the V_____.</v>
       </c>
     </row>
     <row r="174">
@@ -5444,7 +5444,7 @@
         <v>Blue = live wire, brown = neutral, green/yellow stripes = earth</v>
       </c>
       <c r="I174" t="str">
-        <v>In a UK mains plug, the three wires and their colours are _____.</v>
+        <v>In a UK plug: b_____ = neutral, b_____ = live, g_____/y_____ stripes = earth.</v>
       </c>
     </row>
     <row r="175">
@@ -5473,7 +5473,7 @@
         <v>insulation on live and neutral prongs, cable grip to prevent cable being pulled loose, fuse, colour coded wires to prevent confusion, Earth pin and wire</v>
       </c>
       <c r="I175" t="str">
-        <v>Three safety features of a UK mains plug include _____.</v>
+        <v>Three safety features of a UK plug: i_____ on the prongs, a c_____ g_____ and a f_____.</v>
       </c>
     </row>
     <row r="176">
@@ -5502,7 +5502,7 @@
         <v>To melt and break the circuit if too much current flows.</v>
       </c>
       <c r="I176" t="str">
-        <v>A mains plug needs a fuse to _____.</v>
+        <v>A mains plug needs a f_____ to melt and break the circuit if too much current flows.</v>
       </c>
     </row>
     <row r="177">
@@ -5531,7 +5531,7 @@
         <v>A force that acts when objects are physically touching</v>
       </c>
       <c r="I177" t="str">
-        <v>A contact force is _____.</v>
+        <v>A force that only acts when two objects are physically t_____ is called a c_____ f_____.</v>
       </c>
     </row>
     <row r="178">
@@ -5560,7 +5560,7 @@
         <v>A push or a pull that acts on an object due to the interaction with another object</v>
       </c>
       <c r="I178" t="str">
-        <v>A force is _____.</v>
+        <v>A push or pull that acts on an object due to an interaction is called a f_____.</v>
       </c>
     </row>
     <row r="179">
@@ -5589,7 +5589,7 @@
         <v>A force that acts when objects are physically separated</v>
       </c>
       <c r="I179" t="str">
-        <v>A non-contact force is _____.</v>
+        <v>A force that can act between objects without them needing to touch is called a n_____-c_____ f_____.</v>
       </c>
     </row>
     <row r="180">
@@ -5618,7 +5618,7 @@
         <v>Push force acting between two solid objects</v>
       </c>
       <c r="I180" t="str">
-        <v>Normal contact force is _____.</v>
+        <v>The push force that acts perpendicularly between two solid objects in contact is called the n_____ c_____ f_____.</v>
       </c>
     </row>
     <row r="181">
@@ -5647,7 +5647,7 @@
         <v>Force squashing or pushing together</v>
       </c>
       <c r="I181" t="str">
-        <v>Compression is _____.</v>
+        <v>A force that squashes or pushes objects together is called c_____.</v>
       </c>
     </row>
     <row r="182">
@@ -5676,7 +5676,7 @@
         <v>Force extending or pulling apart</v>
       </c>
       <c r="I182" t="str">
-        <v>Tension is _____.</v>
+        <v>A force that stretches or pulls an object apart is called t_____.</v>
       </c>
     </row>
     <row r="183">
@@ -5705,7 +5705,7 @@
         <v>The force at which an object ceases behaving elastically (returns to original shape) and starts behaving plastically (permanent deformation)</v>
       </c>
       <c r="I183" t="str">
-        <v>The elastic limit is _____.</v>
+        <v>The point at which a material permanently deforms and stops returning to its original shape is the e_____ l_____.</v>
       </c>
     </row>
     <row r="184">
@@ -5734,7 +5734,7 @@
         <v>Newton meter</v>
       </c>
       <c r="I184" t="str">
-        <v>Forces are measured using a _____.</v>
+        <v>Forces are measured using a N_____ m_____.</v>
       </c>
     </row>
     <row r="185">
@@ -5763,7 +5763,7 @@
         <v>Friction force acting between an object and air particles</v>
       </c>
       <c r="I185" t="str">
-        <v>Air resistance is _____.</v>
+        <v>The friction force acting on an object as it moves through the air is called a_____ r_____.</v>
       </c>
     </row>
     <row r="186">
@@ -5792,7 +5792,7 @@
         <v>Friction force when one object is a liquid or a gas</v>
       </c>
       <c r="I186" t="str">
-        <v>Drag is _____.</v>
+        <v>The friction force acting on an object moving through a liquid or gas is called d_____.</v>
       </c>
     </row>
     <row r="187">
@@ -5821,7 +5821,7 @@
         <v>Force opposing motion which is caused by the interaction of surfaces moving over each other</v>
       </c>
       <c r="I187" t="str">
-        <v>Friction is _____.</v>
+        <v>The force that opposes motion between two surfaces in contact is called f_____.</v>
       </c>
     </row>
     <row r="188">
@@ -5850,7 +5850,7 @@
         <v>Sports, vehicles</v>
       </c>
       <c r="I188" t="str">
-        <v>Two situations where it is useful to reduce friction are _____.</v>
+        <v>Two situations where reducing friction is useful: in s_____ and in v_____.</v>
       </c>
     </row>
     <row r="189">
@@ -5879,7 +5879,7 @@
         <v>It decreases</v>
       </c>
       <c r="I189" t="str">
-        <v>Increasing the surface area of shoes _____ the pressure exerted on the ground.</v>
+        <v>Increasing the surface area of shoes d_____ the pressure exerted on the ground.</v>
       </c>
     </row>
     <row r="190">
@@ -5908,7 +5908,7 @@
         <v>Pressure = Force/Area</v>
       </c>
       <c r="I190" t="str">
-        <v>The equation for calculating pressure is _____.</v>
+        <v>The equation for pressure is: P = F ÷ _____.</v>
       </c>
     </row>
     <row r="191">
@@ -5937,7 +5937,7 @@
         <v>Pascal, Pa (accept N/m^2 or N/cm^2)</v>
       </c>
       <c r="I191" t="str">
-        <v>The unit of pressure is _____.</v>
+        <v>The unit of pressure is the P_____ (Pa).</v>
       </c>
     </row>
     <row r="192">
@@ -5966,7 +5966,7 @@
         <v>Single force that can replace all the forces acting on an object and have the same effect</v>
       </c>
       <c r="I192" t="str">
-        <v>The resultant force is _____.</v>
+        <v>The single force that has the same effect as all individual forces combined is called the r_____ f_____.</v>
       </c>
     </row>
     <row r="193">
@@ -5995,7 +5995,7 @@
         <v>Object accelerates (speeds up), decelerates (slows down), changes shape, changes direction</v>
       </c>
       <c r="I193" t="str">
-        <v>When forces on an object are unbalanced, the object could _____.</v>
+        <v>When forces are unbalanced, an object may a_____, d_____, change s_____ or change d_____.</v>
       </c>
     </row>
     <row r="194">
@@ -6024,7 +6024,7 @@
         <v>Object remains at rest, object remains at constant speed and direction</v>
       </c>
       <c r="I194" t="str">
-        <v>When forces on an object are balanced, the object _____.</v>
+        <v>When forces are balanced, an object either stays at r_____ or moves at c_____ s_____.</v>
       </c>
     </row>
     <row r="195">
@@ -6053,7 +6053,7 @@
         <v>Zero</v>
       </c>
       <c r="I195" t="str">
-        <v>If forces on an object are balanced, the resultant force is _____.</v>
+        <v>If all forces on an object are balanced, the resultant force is _____.</v>
       </c>
     </row>
     <row r="196">
@@ -6082,7 +6082,7 @@
         <v>The maximum vibration, measured from the middle position of the wave</v>
       </c>
       <c r="I196" t="str">
-        <v>Amplitude is _____.</v>
+        <v>The maximum displacement of a wave from its resting position is called its a_____.</v>
       </c>
     </row>
     <row r="197">
@@ -6111,7 +6111,7 @@
         <v>Number of waves produced per second, in Hertz</v>
       </c>
       <c r="I197" t="str">
-        <v>Frequency is _____.</v>
+        <v>The number of complete waves produced per second, measured in Hertz, is called f_____.</v>
       </c>
     </row>
     <row r="198">
@@ -6140,7 +6140,7 @@
         <v>How high or low the sound is.A high pitch has a high frequency.</v>
       </c>
       <c r="I198" t="str">
-        <v>The pitch of a sound wave refers to _____.</v>
+        <v>The p_____ of a sound (how high or low it sounds) is determined by its f_____.</v>
       </c>
     </row>
     <row r="199">
@@ -6169,7 +6169,7 @@
         <v>How loud or quiet a sound is. A high volume has a high amplitude.</v>
       </c>
       <c r="I199" t="str">
-        <v>The volume of a sound wave refers to _____.</v>
+        <v>The v_____ of a sound (how loud or quiet it is) is determined by its a_____.</v>
       </c>
     </row>
     <row r="200">
@@ -6198,7 +6198,7 @@
         <v>The mid-point of a wave vibration</v>
       </c>
       <c r="I200" t="str">
-        <v>The resting point (rarefaction) of a wave is _____.</v>
+        <v>The mid-point of a wave's vibration, where particles return to rest, is called the r_____ p_____.</v>
       </c>
     </row>
     <row r="201">
@@ -6227,7 +6227,7 @@
         <v>A space with no particles in it</v>
       </c>
       <c r="I201" t="str">
-        <v>A vacuum is _____.</v>
+        <v>A region of space that contains no matter or particles at all is called a v_____.</v>
       </c>
     </row>
     <row r="202">
@@ -6256,7 +6256,7 @@
         <v>330m/s</v>
       </c>
       <c r="I202" t="str">
-        <v>The speed of sound in air is _____.</v>
+        <v>The speed of sound in air is _____ m/s.</v>
       </c>
     </row>
     <row r="203">
@@ -6285,7 +6285,7 @@
         <v>v=fλ, wave speed = frequency x wavelength</v>
       </c>
       <c r="I203" t="str">
-        <v>The wave equation for speed is _____.</v>
+        <v>The wave equation is: wave speed = f_____ × w_____.</v>
       </c>
     </row>
     <row r="204">
@@ -6314,7 +6314,7 @@
         <v>The range of frequencies that an animal can hear (for humans 20Hz to 20000Hz)</v>
       </c>
       <c r="I204" t="str">
-        <v>Auditory range is _____.</v>
+        <v>The range of sound frequencies that an organism can detect is called its a_____ r_____.</v>
       </c>
     </row>
     <row r="205">
@@ -6343,7 +6343,7 @@
         <v>Sound waves with frequency higher than the auditory range</v>
       </c>
       <c r="I205" t="str">
-        <v>Ultrasound refers to _____.</v>
+        <v>Sound waves with a frequency above the human hearing range are called u_____.</v>
       </c>
     </row>
     <row r="206">
@@ -6372,7 +6372,7 @@
         <v>Ear drum, bones, cochlea, auditory nerve, semi-circular canals, pinner</v>
       </c>
       <c r="I206" t="str">
-        <v>The six parts of the ear are _____.</v>
+        <v>The six parts of the ear: e_____ d_____, b_____, c_____, a_____ n_____, s_____-c_____ c_____ and p_____.</v>
       </c>
     </row>
     <row r="207">
@@ -6401,7 +6401,7 @@
         <v>Hammer, anvil, stirrup</v>
       </c>
       <c r="I207" t="str">
-        <v>The three bones in the middle ear are _____.</v>
+        <v>The three tiny bones in the middle ear are the h_____, a_____ and s_____.</v>
       </c>
     </row>
     <row r="208">
@@ -6430,7 +6430,7 @@
         <v>A short pulse of sound (usually ultrasound) is emitted. This reflects off neaby objected and some of the sound travels back to the emitter and is detected. Animals and devices can work out the distance an object is away by how long it took until the echo was heard.</v>
       </c>
       <c r="I208" t="str">
-        <v>Echolocation works by _____.</v>
+        <v>Echolocation works by sending out a sound pulse that r_____ off objects — the return time reveals the d_____.</v>
       </c>
     </row>
     <row r="209">
@@ -6459,7 +6459,7 @@
         <v>It can detect when predators such as bats are nearby.</v>
       </c>
       <c r="I209" t="str">
-        <v>Being able to hear ultrasound benefits moths because _____.</v>
+        <v>Being able to hear u_____ benefits moths (that cannot echolocate) because they can detect predators like b_____.</v>
       </c>
     </row>
     <row r="210">
@@ -6488,7 +6488,7 @@
         <v>The sound could be reflected, absorbed, or transmitted.</v>
       </c>
       <c r="I210" t="str">
-        <v>When sound reaches the interface between two media, it can be _____.</v>
+        <v>When sound reaches the boundary between two media, it can be r_____, a_____ or t_____.</v>
       </c>
     </row>
     <row r="211">
@@ -6517,7 +6517,7 @@
         <v>A wave where the direction of vibration is parallel to the direction the wave travels</v>
       </c>
       <c r="I211" t="str">
-        <v>In a longitudinal wave, _____.</v>
+        <v>In a longitudinal wave, the direction of vibration is p_____ to the direction the wave travels.</v>
       </c>
     </row>
     <row r="212">
@@ -6546,7 +6546,7 @@
         <v>A wave where the direction of vibration is perpendicular/at right angles to the direction the wave travels.</v>
       </c>
       <c r="I212" t="str">
-        <v>In a transverse wave, _____.</v>
+        <v>In a transverse wave, the direction of vibration is p_____ (at right angles) to the direction the wave travels.</v>
       </c>
     </row>
     <row r="213">
@@ -6575,7 +6575,7 @@
         <v>Superposition</v>
       </c>
       <c r="I213" t="str">
-        <v>When two waves overlap, we say they are in _____.</v>
+        <v>When two waves overlap, we say they are in s_____.</v>
       </c>
     </row>
     <row r="214">
@@ -6604,7 +6604,7 @@
         <v>Proteins</v>
       </c>
       <c r="I214" t="str">
-        <v>Biuret solution is used to test for _____.</v>
+        <v>Biuret solution is used to test for p_____.</v>
       </c>
     </row>
     <row r="215">
@@ -6633,7 +6633,7 @@
         <v>Carbohydrates, proteins, fats, fibre, vitamins, minerals, water</v>
       </c>
       <c r="I215" t="str">
-        <v>The 7 food groups are _____.</v>
+        <v>The 7 food groups: c_____, p_____, f_____, f_____, v_____, m_____ and w_____.</v>
       </c>
     </row>
     <row r="216">
@@ -6662,7 +6662,7 @@
         <v>Fats</v>
       </c>
       <c r="I216" t="str">
-        <v>Lipids is another name for _____.</v>
+        <v>Lipids is another name for f_____.</v>
       </c>
     </row>
     <row r="217">
@@ -6691,7 +6691,7 @@
         <v>Rice and pasta</v>
       </c>
       <c r="I217" t="str">
-        <v>Two examples of foods rich in carbohydrates are _____.</v>
+        <v>Two examples of foods rich in carbohydrates are r_____ and p_____.</v>
       </c>
     </row>
     <row r="218">
@@ -6720,7 +6720,7 @@
         <v>Brown bread and cereal</v>
       </c>
       <c r="I218" t="str">
-        <v>Two examples of foods rich in fibre are _____.</v>
+        <v>Two examples of foods rich in fibre are b_____ b_____ and c_____.</v>
       </c>
     </row>
     <row r="219">
@@ -6749,7 +6749,7 @@
         <v>Butter, cheese and chocolate</v>
       </c>
       <c r="I219" t="str">
-        <v>Three examples of foods rich in fat are _____.</v>
+        <v>Three examples of foods rich in fat are b_____, c_____ and c_____.</v>
       </c>
     </row>
     <row r="220">
@@ -6778,7 +6778,7 @@
         <v>Fruit and vegetables</v>
       </c>
       <c r="I220" t="str">
-        <v>Examples of foods rich in minerals and vitamins include _____.</v>
+        <v>Foods rich in minerals and vitamins include f_____ and v_____.</v>
       </c>
     </row>
     <row r="221">
@@ -6807,7 +6807,7 @@
         <v>Refusing to eat to lose weight</v>
       </c>
       <c r="I221" t="str">
-        <v>Anorexia is _____.</v>
+        <v>An eating disorder where a person severely restricts food intake to lose weight is called a_____.</v>
       </c>
     </row>
     <row r="222">
@@ -6836,7 +6836,7 @@
         <v>Eating a variety of foods in the correct proportions</v>
       </c>
       <c r="I222" t="str">
-        <v>A balanced diet is _____.</v>
+        <v>Eating the right variety and amounts of each food group is called a b_____ d_____.</v>
       </c>
     </row>
     <row r="223">
@@ -6865,7 +6865,7 @@
         <v>1) very active, 2) growing, 3) pregnant</v>
       </c>
       <c r="I223" t="str">
-        <v>Three reasons why someone may need more calories than normal include being _____.</v>
+        <v>Three reasons for needing more calories: being very a_____, g_____, or being p_____.</v>
       </c>
     </row>
     <row r="224">
@@ -6894,7 +6894,7 @@
         <v>Obesity, anorexia and Type 2 diabetes</v>
       </c>
       <c r="I224" t="str">
-        <v>Three diseases associated with an unbalanced diet are _____.</v>
+        <v>Three diseases associated with an unbalanced diet: o_____, a_____ and type 2 d_____.</v>
       </c>
     </row>
     <row r="225">
@@ -6923,7 +6923,7 @@
         <v>Mouth, oesophagus, stomach, pancreas, liver, small intestine, large intestine</v>
       </c>
       <c r="I225" t="str">
-        <v>The 7 main organs of the digestive system are _____.</v>
+        <v>The 7 main organs of the digestive system: m_____, o_____, s_____, p_____, l_____, s_____ i_____ and l_____ i_____.</v>
       </c>
     </row>
     <row r="226">
@@ -6952,7 +6952,7 @@
         <v>Water</v>
       </c>
       <c r="I226" t="str">
-        <v>_____ is absorbed from the large intestine.</v>
+        <v>W_____ is absorbed from the large intestine.</v>
       </c>
     </row>
     <row r="227">
@@ -6981,7 +6981,7 @@
         <v>Nutrients</v>
       </c>
       <c r="I227" t="str">
-        <v>_____ are absorbed from the small intestine.</v>
+        <v>N_____ are absorbed from the small intestine.</v>
       </c>
     </row>
     <row r="228">
@@ -7010,7 +7010,7 @@
         <v>Amino acids</v>
       </c>
       <c r="I228" t="str">
-        <v>When proteins are digested, _____ are produced.</v>
+        <v>When proteins are digested, a_____ a_____ are produced.</v>
       </c>
     </row>
     <row r="229">
@@ -7039,7 +7039,7 @@
         <v>Particles travel from areas of high concentration to areas of lower concentration until they are evenly spread out.</v>
       </c>
       <c r="I229" t="str">
-        <v>Diffusion is when _____.</v>
+        <v>The spreading of particles from high to low concentration until evenly spread is called d_____.</v>
       </c>
     </row>
     <row r="230">
@@ -7068,7 +7068,7 @@
         <v>Villi</v>
       </c>
       <c r="I230" t="str">
-        <v>The small intestine has a large surface area because of _____.</v>
+        <v>The small intestine has a large surface area due to tiny finger-like projections called v_____.</v>
       </c>
     </row>
     <row r="231">
@@ -7097,7 +7097,7 @@
         <v>Thin cell walls, a network of capillaries and a large surface area.</v>
       </c>
       <c r="I231" t="str">
-        <v>Villi aid nutrient absorption because they have _____.</v>
+        <v>Villi aid absorption because they have t_____ c_____ w_____, a network of c_____ and a large s_____ a_____.</v>
       </c>
     </row>
     <row r="232">
@@ -7126,7 +7126,7 @@
         <v>Physical changes do not involve chemical reactions, and can often be reversed</v>
       </c>
       <c r="I232" t="str">
-        <v>Unlike chemical changes, physical changes _____.</v>
+        <v>Unlike chemical changes, physical changes do not involve a chemical r_____ and can often be r_____.</v>
       </c>
     </row>
     <row r="233">
@@ -7155,7 +7155,7 @@
         <v>Physical change</v>
       </c>
       <c r="I233" t="str">
-        <v>Evaporation is a _____ change.</v>
+        <v>Evaporation is a p_____ change — no new substances are created.</v>
       </c>
     </row>
     <row r="234">
@@ -7184,7 +7184,7 @@
         <v>All matter is made up of indestructable atoms, which cannot be created or destroyed. Atoms in an element are identical to one another, but each element is made up of a different atom.</v>
       </c>
       <c r="I234" t="str">
-        <v>Dalton's atomic model stated that _____.</v>
+        <v>Dalton's atomic model stated all matter is made of indestructible a_____, identical within each e_____.</v>
       </c>
     </row>
     <row r="235">
@@ -7213,7 +7213,7 @@
         <v>CH4</v>
       </c>
       <c r="I235" t="str">
-        <v>Carbon hydride with a 1:4 ratio of carbon to hydrogen has the formula _____.</v>
+        <v>Carbon hydride with a 1:4 carbon-to-hydrogen ratio has the formula _____.</v>
       </c>
     </row>
     <row r="236">
@@ -7242,7 +7242,7 @@
         <v>1:2</v>
       </c>
       <c r="I236" t="str">
-        <v>In carbon dioxide, the ratio of carbon to oxygen atoms is _____.</v>
+        <v>In carbon dioxide (CO₂), the ratio of carbon to oxygen atoms is _____.</v>
       </c>
     </row>
     <row r="237">
@@ -7271,7 +7271,7 @@
         <v>5g</v>
       </c>
       <c r="I237" t="str">
-        <v>When 4g of zinc reacts completely with 1g of oxygen, _____ of zinc oxide is produced.</v>
+        <v>When 4g of zinc reacts with 1g of oxygen, conservation of mass means _____ g of zinc oxide is produced.</v>
       </c>
     </row>
     <row r="238">
@@ -7300,7 +7300,7 @@
         <v>Columns in the periodic table</v>
       </c>
       <c r="I238" t="str">
-        <v>In the periodic table, a group is _____.</v>
+        <v>The vertical columns in the periodic table are called g_____.</v>
       </c>
     </row>
     <row r="239">
@@ -7329,7 +7329,7 @@
         <v>In order of atomic number (lowest to highest)</v>
       </c>
       <c r="I239" t="str">
-        <v>Elements in the periodic table are arranged _____.</v>
+        <v>Elements in the periodic table are arranged in order of increasing a_____ n_____.</v>
       </c>
     </row>
     <row r="240">
@@ -7358,7 +7358,7 @@
         <v>Use the atomic number</v>
       </c>
       <c r="I240" t="str">
-        <v>The number of electrons in an element equals _____.</v>
+        <v>The number of electrons in a neutral atom equals its a_____ n_____.</v>
       </c>
     </row>
     <row r="241">
@@ -7387,7 +7387,7 @@
         <v>Mass number - atomic number</v>
       </c>
       <c r="I241" t="str">
-        <v>The number of neutrons in an element is calculated by _____.</v>
+        <v>Number of neutrons = m_____ n_____ − a_____ n_____.</v>
       </c>
     </row>
     <row r="242">
@@ -7416,7 +7416,7 @@
         <v>Rows in the periodic table</v>
       </c>
       <c r="I242" t="str">
-        <v>In the periodic table, a period is _____.</v>
+        <v>The horizontal rows in the periodic table are called p_____.</v>
       </c>
     </row>
     <row r="243" xml:space="preserve">
@@ -7448,7 +7448,7 @@
  *Malleable</v>
       </c>
       <c r="I243" t="str">
-        <v>Four properties of metals include _____.</v>
+        <v>Four properties of metals: h_____ m_____ point, good c_____, d_____ and m_____.</v>
       </c>
     </row>
     <row r="244" xml:space="preserve">
@@ -7479,7 +7479,7 @@
  *Brittle</v>
       </c>
       <c r="I244" t="str">
-        <v>Four properties of non-metals include _____.</v>
+        <v>Four properties of non-metals: l_____ m_____ point, b_____ when solid, not s_____, poor c_____.</v>
       </c>
     </row>
     <row r="245">
@@ -7508,7 +7508,7 @@
         <v>Astatine, Iodine, Bromine, Chlorine, Fluorine</v>
       </c>
       <c r="I245" t="str">
-        <v>The 5 halogens in order of reactivity from lowest to highest are _____.</v>
+        <v>The 5 halogens, lowest to highest reactivity: a_____, i_____, b_____, c_____, f_____.</v>
       </c>
     </row>
     <row r="246">
@@ -7537,7 +7537,7 @@
         <v>Lithium, sodium, potassium, rubidium, caesium, francium</v>
       </c>
       <c r="I246" t="str">
-        <v>The 6 alkali metals in order of reactivity from lowest to highest are _____.</v>
+        <v>The 6 alkali metals, lowest to highest reactivity: l_____, s_____, p_____, r_____, c_____, f_____.</v>
       </c>
     </row>
     <row r="247">
@@ -7566,7 +7566,7 @@
         <v>Increases</v>
       </c>
       <c r="I247" t="str">
-        <v>As you move down group 1 (alkali metals), reactivity _____.</v>
+        <v>As you move down group 1, reactivity i_____.</v>
       </c>
     </row>
     <row r="248">
@@ -7595,7 +7595,7 @@
         <v>Alkaline metal hydroxide</v>
       </c>
       <c r="I248" t="str">
-        <v>When alkali metals react with water, _____ is formed.</v>
+        <v>When alkali metals react with water, m_____ h_____ is formed (plus hydrogen gas).</v>
       </c>
     </row>
     <row r="249">
@@ -7624,7 +7624,7 @@
         <v>Shiny</v>
       </c>
       <c r="I249" t="str">
-        <v>When freshly cut, alkali metals appear _____.</v>
+        <v>When freshly cut, alkali metals appear s_____.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>